<commit_message>
docs(P0): wy-worklog.com 도메인 연결 기록·재검증 결과 (D-55)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/P0-화면테스트_v1.0.xlsx
+++ b/docs/qa/P0-화면테스트_v1.0.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="테스트 항목" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="범위 밖" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="도메인 전환 재검증" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'테스트 항목'!$A$1:$L$63</definedName>
@@ -4788,7 +4789,529 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>없음 (FAIL 0). 문서 대조 관찰 4건은 각 TC 비고 참고: TC-39 토스트 [다시 시도] 없음, TC-73 모바일 띠 '재시도 중…' 표시, TC-74 오류 페이지 '입력한 내용은 저장되어 있어요' 문구, TC-81 '다시 로그인해 주세요' 안내는 P0 화면에서 재현 불가 / 재검증 2026-10-05: ErrorPage 본문 수정 후 TC-74·76·79 PASS(로컬, 점검 화면 문구 변경 없음 확인)</t>
+          <t>없음 (FAIL 0). 문서 대조 관찰 4건은 각 TC 비고 참고: TC-39 토스트 [다시 시도] 없음, TC-73 모바일 띠 '재시도 중…' 표시, TC-74 오류 페이지 '입력한 내용은 저장되어 있어요' 문구, TC-81 '다시 로그인해 주세요' 안내는 P0 화면에서 재현 불가 / 재검증 2026-10-05: ErrorPage 본문 수정 후 TC-74·76·79 PASS(로컬, 점검 화면 문구 변경 없음 확인) / 도메인 전환 재검증 2026-10-05(https://wy-worklog.com): 10항목 PASS, 결함 없음 → '도메인 전환 재검증' 시트</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>관련 TC</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>확인 항목</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>절차</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>기대 결과</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>실제 결과</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>판정</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>증거(스크린샷 경로)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>비고</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>DOM-01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>TC-01</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>가입(www에서 시작)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.wy-worklog.com/signup 접속 → 새 qa- 계정으로 가입</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>apex로 308 후 가입 201, 홈 이동</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>www → https://wy-worklog.com/signup 이동, POST /api/auth/signup 201, 홈(/) 이동</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>C:/Users/ksoun/AppData/Local/Temp/claude/c--projects-erp-project/e57b7bdc-5748-46c9-aff5-11c4a94b9d55/scratchpad/shots/DOM-signup-home.png</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>도메인 전환 재검증 2026-10-05. 계정 qa-dom-10052307@example.com (23:07 가입)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>DOM-02</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>TC-02, TC-03</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>로그인 → 인증 API</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>새 도메인에서 로그인(curl, Origin=https://wy-worklog.com), 브라우저에서 GET /api/users/me</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>로그인 200, me 200</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>로그인 200, 브라우저 me 200(본인 email, x-vercel-cache MISS)</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>도메인 전환 재검증 2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>DOM-03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>TC-04, TC-05</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>새로고침·새 탭 유지</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>/calendar 새로고침, 새 탭으로 /stats·/logs</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>로그인 유지</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>새로고침 후 me 200·/calendar 유지, 새 탭(t3) /stats '통계' 표시</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>C:/Users/ksoun/AppData/Local/Temp/claude/c--projects-erp-project/e57b7bdc-5748-46c9-aff5-11c4a94b9d55/scratchpad/shots/DOM-newtab.png</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>도메인 전환 재검증 2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>DOM-04</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>TC-06</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>토큰 자동 갱신</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>가입 10분 뒤(access 만료) /tasks 새로고침</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>me 401 → refresh → me 200, 화면 유지</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>23:18 새로고침: GET /api/users/me 401 → POST /api/auth/refresh 204 → GET /api/users/me 200, '업무' 화면 유지</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>C:/Users/ksoun/AppData/Local/Temp/claude/c--projects-erp-project/e57b7bdc-5748-46c9-aff5-11c4a94b9d55/scratchpad/shots/DOM-refresh.png</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>도메인 전환 재검증 2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>DOM-05</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>TC-93</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>쿠키 속성·도메인</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>로그인 응답 Set-Cookie와 curl cookie jar 확인</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>HttpOnly·Secure·SameSite=Strict, 쿠키 도메인 wy-worklog.com</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>access_token(Path=/api, 600초)·refresh_token(Path=/api/auth, 14일) 모두 Secure; HttpOnly; SameSite=Strict, Domain 속성 없음 → host-only wy-worklog.com(서브도메인 미공유). document.cookie 빈 문자열</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>도메인 전환 재검증 2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>DOM-06</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>www·http → apex 308</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>curl: https://www.wy-worklog.com/, /stats?x=1, POST /api/auth/login, http://wy-worklog.com/</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>모두 apex https로 308(경로·쿼리 유지), 이후 정상 로그인</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>모두 308, Location이 https://wy-worklog.com + 원래 경로·쿼리. www에서 시작한 가입·로그인 흐름 정상(DOM-01)</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>도메인 전환 재검증 2026-10-05. 인증서 CN=wy-worklog.com(Let's Encrypt, 2027-01-03 만료), HSTS max-age=63072000</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>DOM-07</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>TC-90~92</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>다른 Origin 쓰기 403</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>새 도메인 POST /api/auth/login에 Origin을 evil·www·http·없음·옛 vercel.app으로</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>허용 목록 외 403 ORIGIN_REJECTED</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>evil.example.com·https://www.wy-worklog.com·http://wy-worklog.com·Origin 없음 → 403 ORIGIN_REJECTED. https://project-7qtt1.vercel.app → 통과(401 INVALID_CREDENTIALS)</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>도메인 전환 재검증 2026-10-05. 옛 도메인 Origin 허용은 전환 기간 유지 방침대로. 옛 도메인 폐기 때 ALLOWED_ORIGINS에서 빼야 함</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>DOM-08</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>TC-102, TC-103</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>x-vercel-cache 비 HIT</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>/api/users/me 3회 + 브라우저 API 응답 확인</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>HIT 아님</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>API 응답 전부 MISS, X-Trace-Id = 본문 traceId</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>도메인 전환 재검증 2026-10-05. 정적 페이지 / 는 HIT(정적 파일 캐시라 정상)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>DOM-09</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>TC-52, TC-60, TC-61</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>390px 레이아웃</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>폭 390px로 앱 셸·/login·/signup</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>가로 스크롤 없음, 하단 탭 화면 안</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>세 화면 scrollWidth 390, 넘치는 요소 0, 사이드바 숨김·하단 탭 bottom=844</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>C:/Users/ksoun/AppData/Local/Temp/claude/c--projects-erp-project/e57b7bdc-5748-46c9-aff5-11c4a94b9d55/scratchpad/shots/DOM-390-shell.png</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>도메인 전환 재검증 2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>DOM-10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>TC-02</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>옛 도메인 로그인(전환 기간)</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>https://project-7qtt1.vercel.app/login에서 기존 qa 계정 로그인 후 새로고침</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>로그인 200, 유지</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>POST /api/auth/login 200, 홈 이동, 새로고침 후 유지</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>C:/Users/ksoun/AppData/Local/Temp/claude/c--projects-erp-project/e57b7bdc-5748-46c9-aff5-11c4a94b9d55/scratchpad/shots/DOM-old-login.png</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>도메인 전환 재검증 2026-10-05. 옛 도메인 세션으로 wy-worklog.com 접속 시 /login(쿠키가 도메인별이라 세션 미공유, 정상)</t>
         </is>
       </c>
     </row>

</xml_diff>